<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@4d5adb341372023e0addaf55127c2f800f5efd0d 🚀
</commit_message>
<xml_diff>
--- a/behandelaanwijzing-2017-2020.xlsx
+++ b/behandelaanwijzing-2017-2020.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t>Property</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-21T07:57:06+00:00</t>
+    <t>2024-02-21T09:14:14+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -112,6 +112,9 @@
     <t>Relationship</t>
   </si>
   <si>
+    <t>2.16.840.1.113883.2.4.3.11.60.40.3.2.2</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -137,6 +140,9 @@
   </si>
   <si>
     <t>Toelichting</t>
+  </si>
+  <si>
+    <t>urn:oid:2.16.840.1.113883.2.4.3.11.60.40.4.25.1</t>
   </si>
   <si>
     <t>JA</t>
@@ -473,67 +479,69 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2"/>
+      <c r="A2" t="s" s="2">
+        <v>32</v>
+      </c>
       <c r="B2" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -565,67 +573,69 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2"/>
+      <c r="A2" t="s" s="2">
+        <v>42</v>
+      </c>
       <c r="B2" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>